<commit_message>
nuevo input para plantilla productos
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_productos.xlsx
+++ b/frontend/public/plantilla_productos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferna\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\fer\drogueria-virtual\frontend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B2BA6E7-9ED7-4162-812E-D5E49AE03952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86B65A4-3304-42A1-A944-DB3D1ADB72F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Productos" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>NombreProducto</t>
   </si>
@@ -67,9 +67,6 @@
     <t>ViaAdministracion</t>
   </si>
   <si>
-    <t>RegistroISP (1=Sí, 0=No)</t>
-  </si>
-  <si>
     <t>Precio</t>
   </si>
   <si>
@@ -116,6 +113,12 @@
   </si>
   <si>
     <t>Oral</t>
+  </si>
+  <si>
+    <t>RegistroISP</t>
+  </si>
+  <si>
+    <t>REGISTRO-32P38943</t>
   </si>
 </sst>
 </file>
@@ -125,7 +128,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +148,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -174,7 +183,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -186,54 +195,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -535,7 +509,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -551,7 +525,7 @@
     <col min="13" max="13" width="9" customWidth="1"/>
     <col min="14" max="14" width="7" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="26" customWidth="1"/>
+    <col min="16" max="16" width="26" style="9" customWidth="1"/>
     <col min="17" max="17" width="8" style="3" customWidth="1"/>
     <col min="18" max="18" width="7" style="4" customWidth="1"/>
   </cols>
@@ -602,81 +576,77 @@
       <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="R1" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="R1" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="G2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="H2" s="7">
+        <v>46387</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="13">
-        <v>46387</v>
-      </c>
-      <c r="I2" s="14" t="s">
+      <c r="J2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="K2" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="N2" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="O2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="O2" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="20">
+      <c r="P2" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="6">
         <v>5.99</v>
       </c>
-      <c r="R2" s="21">
+      <c r="R2" s="6">
         <v>150</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="P2:P500" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>"0,1"</formula1>
-    </dataValidation>
-  </dataValidations>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1" xr:uid="{493CF628-AC12-43DC-8D87-819C428EC469}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>